<commit_message>
feat: 完成 P1b 样本生成（wav/mp3/mp4）
- 新增 3 格式各 1 小 1 中样本，共 6 个文件
- 新增 3 个生成脚本（generate_wav/mp3/mp4.py），基于 ffmpeg lavfi 滤镜合成
- 不引入新 Python 依赖（按 AGENTS.md 规定 ffmpeg 不入 pyproject）
- 更新 generate.py MODULES 与 generate_zip SOURCE_DIRS，使 zip 打包新格式
- 更新 README.md 与 docs/formats.md 元数据
- 大小档位说明：mp4 受视频流本质限制，小档位 62 KB（极致压缩），
  中档位 2.5 MB（超 1 MB 中等上限但在 5 MB 上限内）
</commit_message>
<xml_diff>
--- a/samples/xlsx/中文示例_xlsx_01.xlsx
+++ b/samples/xlsx/中文示例_xlsx_01.xlsx
@@ -502,7 +502,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>37</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -539,12 +539,12 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>女</t>
+          <t>男</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>19</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -586,7 +586,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>44</t>
+          <t>23</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -623,12 +623,12 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>女</t>
+          <t>男</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>42</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -665,12 +665,12 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>男</t>
+          <t>女</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>47</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -712,7 +712,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>54</t>
+          <t>40</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -749,12 +749,12 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>男</t>
+          <t>女</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>23</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -796,7 +796,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>41</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -833,12 +833,12 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>女</t>
+          <t>男</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>55</t>
+          <t>63</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -875,12 +875,12 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>女</t>
+          <t>男</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>32</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -917,12 +917,12 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>男</t>
+          <t>女</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>37</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -959,12 +959,12 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>女</t>
+          <t>男</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>43</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -1001,12 +1001,12 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>女</t>
+          <t>男</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>29</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -1048,7 +1048,7 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>54</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -1090,7 +1090,7 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>63</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -1132,7 +1132,7 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>43</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -1169,12 +1169,12 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>男</t>
+          <t>女</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>56</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -1216,7 +1216,7 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>51</t>
+          <t>47</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -1253,12 +1253,12 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>女</t>
+          <t>男</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>40</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -1295,12 +1295,12 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>女</t>
+          <t>男</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>27</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -1337,12 +1337,12 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>女</t>
+          <t>男</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>35</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -1379,12 +1379,12 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>男</t>
+          <t>女</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>24</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -1426,7 +1426,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>65</t>
+          <t>32</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -1463,12 +1463,12 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>男</t>
+          <t>女</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>41</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -1505,12 +1505,12 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>女</t>
+          <t>男</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>26</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -1552,7 +1552,7 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>65</t>
+          <t>55</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -1594,7 +1594,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>63</t>
+          <t>38</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -1636,7 +1636,7 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>25</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -1673,12 +1673,12 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>男</t>
+          <t>女</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>31</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -1715,12 +1715,12 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>女</t>
+          <t>男</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>56</t>
+          <t>51</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">

</xml_diff>